<commit_message>
Update to Expo v55
</commit_message>
<xml_diff>
--- a/data/subadapp.xlsx
+++ b/data/subadapp.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="228">
   <si>
     <t xml:space="preserve">no</t>
   </si>
@@ -113,6 +113,9 @@
     <t xml:space="preserve">albumNo</t>
   </si>
   <si>
+    <t xml:space="preserve">album</t>
+  </si>
+  <si>
     <t xml:space="preserve">url</t>
   </si>
   <si>
@@ -188,6 +191,9 @@
     <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/images/thumb/4/4a/%C5%9Eubadap_R.png/300px-%C5%9Eubadap_R.png</t>
   </si>
   <si>
+    <t xml:space="preserve"> Dino'nun Şarkıları</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ben Doğmadan Önce</t>
   </si>
   <si>
@@ -695,25 +701,7 @@
     <t xml:space="preserve">Öcü Möcü Yok Ki! </t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/index.php/%C3%96c%C3%BC_M%C3%B6c%C3%BC_Yok_Ki</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">!</t>
-    </r>
+    <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/index.php/%C3%96c%C3%BC_M%C3%B6c%C3%BC_Yok_Ki!</t>
   </si>
   <si>
     <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/images/9/9a/%C3%96c%C3%BC_M%C3%B6c%C3%BC_Yok_Ki.mp3</t>
@@ -726,7 +714,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -767,15 +755,20 @@
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -829,16 +822,20 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -846,11 +843,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1105,29 +1106,29 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="11.5625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5625" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="28.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="110.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="117.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="110.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="117.56"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1135,16 +1136,16 @@
       <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>2014</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1152,16 +1153,16 @@
       <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>2015</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="2" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1169,16 +1170,16 @@
       <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>2016</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1186,16 +1187,16 @@
       <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>2017</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="2" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1203,16 +1204,16 @@
       <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C6" s="1" t="n">
         <v>2019</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="4" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1220,16 +1221,16 @@
       <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C7" s="1" t="n">
         <v>2020</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" s="2" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1237,16 +1238,16 @@
       <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C8" s="1" t="n">
         <v>2023</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1254,16 +1255,16 @@
       <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C9" s="1" t="n">
         <v>2024</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E9" s="0" t="s">
+      <c r="E9" s="2" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1292,34 +1293,38 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
-  <sheetFormatPr defaultColWidth="11.5625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G52"/>
+  <sheetFormatPr defaultColWidth="11.5625" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3.76"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="102.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="135.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="200.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="28.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="25.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="102.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="135.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="200.11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1330,17 +1335,20 @@
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="D2" s="0" t="s">
+      <c r="C2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>34</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1351,16 +1359,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="D3" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="2" t="s">
         <v>38</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1370,17 +1381,20 @@
       <c r="B4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="0" t="s">
-        <v>39</v>
-      </c>
-      <c r="D4" s="0" t="s">
+      <c r="C4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" s="2" t="s">
         <v>42</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1390,17 +1404,20 @@
       <c r="B5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="0" t="s">
-        <v>43</v>
-      </c>
-      <c r="D5" s="0" t="s">
+      <c r="C5" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" s="2" t="s">
         <v>46</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1410,17 +1427,20 @@
       <c r="B6" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="0" t="s">
-        <v>47</v>
-      </c>
-      <c r="D6" s="0" t="s">
+      <c r="C6" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" s="2" t="s">
         <v>50</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1430,17 +1450,20 @@
       <c r="B7" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="0" t="s">
-        <v>51</v>
-      </c>
-      <c r="D7" s="0" t="s">
+      <c r="C7" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="F7" s="0" t="s">
+      <c r="F7" s="2" t="s">
         <v>54</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1450,17 +1473,20 @@
       <c r="B8" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="D8" s="0" t="s">
+      <c r="C8" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="D8" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="F8" s="0" t="s">
+      <c r="E8" s="2" t="s">
         <v>58</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1470,17 +1496,20 @@
       <c r="B9" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="0" t="s">
-        <v>59</v>
-      </c>
-      <c r="D9" s="0" t="s">
-        <v>60</v>
-      </c>
-      <c r="E9" s="0" t="s">
+      <c r="C9" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F9" s="0" t="s">
+      <c r="E9" s="2" t="s">
         <v>62</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1490,17 +1519,20 @@
       <c r="B10" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="0" t="s">
-        <v>63</v>
-      </c>
-      <c r="D10" s="0" t="s">
-        <v>64</v>
-      </c>
-      <c r="E10" s="0" t="s">
+      <c r="C10" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="E10" s="2" t="s">
         <v>66</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1510,17 +1542,20 @@
       <c r="B11" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C11" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="E11" s="0" t="s">
+      <c r="C11" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F11" s="0" t="s">
+      <c r="E11" s="2" t="s">
         <v>70</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1530,17 +1565,20 @@
       <c r="B12" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="0" t="s">
-        <v>71</v>
-      </c>
-      <c r="D12" s="0" t="s">
-        <v>72</v>
-      </c>
-      <c r="E12" s="0" t="s">
+      <c r="C12" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="F12" s="0" t="s">
+      <c r="E12" s="2" t="s">
         <v>74</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1550,17 +1588,20 @@
       <c r="B13" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="0" t="s">
-        <v>75</v>
-      </c>
-      <c r="D13" s="0" t="s">
-        <v>76</v>
-      </c>
-      <c r="E13" s="0" t="s">
+      <c r="C13" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="F13" s="0" t="s">
+      <c r="E13" s="2" t="s">
         <v>78</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1570,17 +1611,20 @@
       <c r="B14" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="D14" s="0" t="s">
-        <v>80</v>
-      </c>
-      <c r="E14" s="0" t="s">
+      <c r="C14" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="F14" s="0" t="s">
+      <c r="E14" s="2" t="s">
         <v>82</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1590,17 +1634,20 @@
       <c r="B15" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="0" t="s">
-        <v>83</v>
-      </c>
-      <c r="D15" s="0" t="s">
-        <v>84</v>
-      </c>
-      <c r="E15" s="0" t="s">
+      <c r="C15" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F15" s="0" t="s">
+      <c r="E15" s="2" t="s">
         <v>86</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1610,17 +1657,20 @@
       <c r="B16" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C16" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="D16" s="0" t="s">
-        <v>88</v>
-      </c>
-      <c r="E16" s="0" t="s">
+      <c r="C16" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="F16" s="0" t="s">
+      <c r="E16" s="2" t="s">
         <v>90</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1630,17 +1680,20 @@
       <c r="B17" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C17" s="0" t="s">
-        <v>91</v>
-      </c>
-      <c r="D17" s="0" t="s">
-        <v>92</v>
-      </c>
-      <c r="E17" s="0" t="s">
+      <c r="C17" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="F17" s="0" t="s">
+      <c r="E17" s="2" t="s">
         <v>94</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1650,17 +1703,20 @@
       <c r="B18" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C18" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="D18" s="0" t="s">
-        <v>96</v>
-      </c>
-      <c r="E18" s="0" t="s">
+      <c r="C18" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="F18" s="0" t="s">
+      <c r="E18" s="2" t="s">
         <v>98</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1670,17 +1726,20 @@
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C19" s="0" t="s">
-        <v>99</v>
-      </c>
-      <c r="D19" s="0" t="s">
-        <v>100</v>
-      </c>
-      <c r="E19" s="0" t="s">
+      <c r="C19" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F19" s="0" t="s">
+      <c r="E19" s="2" t="s">
         <v>102</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1690,17 +1749,20 @@
       <c r="B20" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C20" s="0" t="s">
-        <v>103</v>
-      </c>
-      <c r="D20" s="0" t="s">
-        <v>104</v>
-      </c>
-      <c r="E20" s="0" t="s">
+      <c r="C20" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="F20" s="0" t="s">
+      <c r="E20" s="2" t="s">
         <v>106</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1710,17 +1772,20 @@
       <c r="B21" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="C21" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D21" s="0" t="s">
-        <v>107</v>
-      </c>
-      <c r="E21" s="0" t="s">
-        <v>108</v>
-      </c>
-      <c r="F21" s="0" t="s">
+      <c r="D21" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>109</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1730,17 +1795,20 @@
       <c r="B22" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C22" s="0" t="s">
-        <v>110</v>
-      </c>
-      <c r="D22" s="0" t="s">
-        <v>111</v>
-      </c>
-      <c r="E22" s="0" t="s">
+      <c r="C22" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="F22" s="0" t="s">
+      <c r="E22" s="2" t="s">
         <v>113</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1750,17 +1818,20 @@
       <c r="B23" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C23" s="0" t="s">
-        <v>114</v>
-      </c>
-      <c r="D23" s="0" t="s">
-        <v>115</v>
-      </c>
-      <c r="E23" s="0" t="s">
+      <c r="C23" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="F23" s="0" t="s">
+      <c r="E23" s="2" t="s">
         <v>117</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1770,17 +1841,20 @@
       <c r="B24" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C24" s="0" t="s">
-        <v>118</v>
-      </c>
-      <c r="D24" s="0" t="s">
-        <v>119</v>
-      </c>
-      <c r="E24" s="0" t="s">
+      <c r="C24" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="F24" s="0" t="s">
+      <c r="E24" s="2" t="s">
         <v>121</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1790,17 +1864,20 @@
       <c r="B25" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C25" s="0" t="s">
-        <v>122</v>
-      </c>
-      <c r="D25" s="0" t="s">
-        <v>123</v>
-      </c>
-      <c r="E25" s="0" t="s">
+      <c r="C25" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F25" s="0" t="s">
+      <c r="E25" s="2" t="s">
         <v>125</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1810,17 +1887,20 @@
       <c r="B26" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C26" s="0" t="s">
-        <v>126</v>
-      </c>
-      <c r="D26" s="0" t="s">
-        <v>127</v>
-      </c>
-      <c r="E26" s="0" t="s">
+      <c r="C26" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="F26" s="0" t="s">
+      <c r="E26" s="2" t="s">
         <v>129</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1830,17 +1910,20 @@
       <c r="B27" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C27" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="D27" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="E27" s="0" t="s">
+      <c r="C27" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="F27" s="0" t="s">
+      <c r="E27" s="2" t="s">
         <v>133</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1850,17 +1933,20 @@
       <c r="B28" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C28" s="0" t="s">
+      <c r="C28" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D28" s="0" t="s">
-        <v>134</v>
-      </c>
-      <c r="E28" s="0" t="s">
-        <v>135</v>
-      </c>
-      <c r="F28" s="0" t="s">
+      <c r="D28" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>136</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1870,17 +1956,20 @@
       <c r="B29" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C29" s="0" t="s">
-        <v>137</v>
-      </c>
-      <c r="D29" s="0" t="s">
-        <v>138</v>
-      </c>
-      <c r="E29" s="0" t="s">
+      <c r="C29" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="F29" s="0" t="s">
+      <c r="E29" s="2" t="s">
         <v>140</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1890,17 +1979,20 @@
       <c r="B30" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C30" s="0" t="s">
-        <v>141</v>
-      </c>
-      <c r="D30" s="0" t="s">
-        <v>142</v>
-      </c>
-      <c r="E30" s="0" t="s">
+      <c r="C30" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F30" s="0" t="s">
+      <c r="E30" s="2" t="s">
         <v>144</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1910,17 +2002,20 @@
       <c r="B31" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C31" s="0" t="s">
-        <v>145</v>
-      </c>
-      <c r="D31" s="0" t="s">
-        <v>146</v>
-      </c>
-      <c r="E31" s="0" t="s">
+      <c r="C31" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="F31" s="0" t="s">
+      <c r="E31" s="2" t="s">
         <v>148</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1930,17 +2025,20 @@
       <c r="B32" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C32" s="0" t="s">
-        <v>149</v>
-      </c>
-      <c r="D32" s="0" t="s">
-        <v>150</v>
-      </c>
-      <c r="E32" s="0" t="s">
+      <c r="C32" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D32" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="F32" s="0" t="s">
+      <c r="E32" s="2" t="s">
         <v>152</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1950,17 +2048,20 @@
       <c r="B33" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C33" s="0" t="s">
+      <c r="C33" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D33" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="E33" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="F33" s="0" t="s">
+      <c r="D33" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>155</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1970,17 +2071,20 @@
       <c r="B34" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C34" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="D34" s="0" t="s">
-        <v>157</v>
-      </c>
-      <c r="E34" s="0" t="s">
+      <c r="C34" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D34" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="F34" s="0" t="s">
+      <c r="E34" s="2" t="s">
         <v>159</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1990,17 +2094,20 @@
       <c r="B35" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C35" s="0" t="s">
-        <v>160</v>
-      </c>
-      <c r="D35" s="0" t="s">
-        <v>161</v>
-      </c>
-      <c r="E35" s="0" t="s">
+      <c r="C35" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="F35" s="0" t="s">
+      <c r="E35" s="2" t="s">
         <v>163</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2010,17 +2117,20 @@
       <c r="B36" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C36" s="0" t="s">
-        <v>164</v>
-      </c>
-      <c r="D36" s="0" t="s">
-        <v>165</v>
-      </c>
-      <c r="E36" s="0" t="s">
+      <c r="C36" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="F36" s="0" t="s">
+      <c r="E36" s="2" t="s">
         <v>167</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2030,17 +2140,20 @@
       <c r="B37" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C37" s="0" t="s">
-        <v>168</v>
-      </c>
-      <c r="D37" s="0" t="s">
-        <v>169</v>
-      </c>
-      <c r="E37" s="0" t="s">
+      <c r="C37" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D37" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="F37" s="0" t="s">
+      <c r="E37" s="2" t="s">
         <v>171</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2050,17 +2163,20 @@
       <c r="B38" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C38" s="0" t="s">
-        <v>172</v>
-      </c>
-      <c r="D38" s="0" t="s">
-        <v>173</v>
-      </c>
-      <c r="E38" s="0" t="s">
+      <c r="C38" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="F38" s="0" t="s">
+      <c r="E38" s="2" t="s">
         <v>175</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2070,17 +2186,20 @@
       <c r="B39" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C39" s="0" t="s">
-        <v>176</v>
-      </c>
-      <c r="D39" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="E39" s="0" t="s">
+      <c r="C39" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="F39" s="0" t="s">
+      <c r="E39" s="2" t="s">
         <v>179</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2090,17 +2209,20 @@
       <c r="B40" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C40" s="0" t="s">
-        <v>180</v>
-      </c>
-      <c r="D40" s="0" t="s">
-        <v>181</v>
-      </c>
-      <c r="E40" s="0" t="s">
+      <c r="C40" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="F40" s="0" t="s">
+      <c r="E40" s="2" t="s">
         <v>183</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2110,17 +2232,20 @@
       <c r="B41" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C41" s="0" t="s">
-        <v>184</v>
-      </c>
-      <c r="D41" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="E41" s="0" t="s">
+      <c r="C41" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D41" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="F41" s="3" t="s">
+      <c r="E41" s="4" t="s">
         <v>187</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2130,17 +2255,20 @@
       <c r="B42" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C42" s="0" t="s">
-        <v>188</v>
-      </c>
-      <c r="D42" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="E42" s="3" t="s">
+      <c r="C42" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D42" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="F42" s="3" t="s">
+      <c r="E42" s="4" t="s">
         <v>191</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2150,17 +2278,20 @@
       <c r="B43" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C43" s="0" t="s">
-        <v>192</v>
-      </c>
-      <c r="D43" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="E43" s="0" t="s">
+      <c r="C43" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D43" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="F43" s="3" t="s">
+      <c r="E43" s="4" t="s">
         <v>195</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2170,17 +2301,20 @@
       <c r="B44" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C44" s="0" t="s">
-        <v>196</v>
-      </c>
-      <c r="D44" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="E44" s="0" t="s">
+      <c r="C44" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D44" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="F44" s="3" t="s">
+      <c r="E44" s="4" t="s">
         <v>199</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="G44" s="4" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2190,17 +2324,20 @@
       <c r="B45" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C45" s="0" t="s">
-        <v>200</v>
-      </c>
-      <c r="D45" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="E45" s="3" t="s">
+      <c r="C45" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="F45" s="3" t="s">
+      <c r="E45" s="4" t="s">
         <v>203</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2210,17 +2347,20 @@
       <c r="B46" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C46" s="0" t="s">
-        <v>204</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="E46" s="3" t="s">
+      <c r="C46" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D46" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="F46" s="3" t="s">
+      <c r="E46" s="4" t="s">
         <v>207</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="G46" s="4" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2230,16 +2370,19 @@
       <c r="B47" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C47" s="0" t="s">
-        <v>208</v>
-      </c>
-      <c r="D47" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="E47" s="4" t="s">
+      <c r="C47" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D47" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="F47" s="5" t="s">
+      <c r="E47" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G47" s="7" t="s">
         <v>28</v>
       </c>
     </row>
@@ -2250,16 +2393,19 @@
       <c r="B48" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C48" s="0" t="s">
-        <v>211</v>
-      </c>
-      <c r="D48" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="E48" s="4" t="s">
+      <c r="C48" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D48" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="F48" s="5" t="s">
+      <c r="E48" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="F48" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="G48" s="7" t="s">
         <v>28</v>
       </c>
     </row>
@@ -2270,16 +2416,19 @@
       <c r="B49" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C49" s="0" t="s">
-        <v>214</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="E49" s="4" t="s">
+      <c r="C49" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D49" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="F49" s="5" t="s">
+      <c r="E49" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="F49" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="G49" s="7" t="s">
         <v>28</v>
       </c>
     </row>
@@ -2290,16 +2439,19 @@
       <c r="B50" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C50" s="0" t="s">
-        <v>217</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="E50" s="4" t="s">
+      <c r="C50" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D50" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="F50" s="5" t="s">
+      <c r="E50" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="F50" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="G50" s="7" t="s">
         <v>28</v>
       </c>
     </row>
@@ -2310,16 +2462,19 @@
       <c r="B51" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C51" s="0" t="s">
-        <v>220</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="E51" s="4" t="s">
+      <c r="C51" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D51" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="F51" s="5" t="s">
+      <c r="E51" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="G51" s="7" t="s">
         <v>28</v>
       </c>
     </row>
@@ -2330,56 +2485,64 @@
       <c r="B52" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C52" s="0" t="s">
-        <v>223</v>
-      </c>
-      <c r="D52" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="E52" s="4" t="s">
+      <c r="C52" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="F52" s="5" t="s">
+      <c r="E52" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="F52" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="G52" s="7" t="s">
         <v>28</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" display="https://ansiklopedi.subadapcocuk.org/images/thumb/e/e9/D%C3%BC%C5%9F-r.png/300px-D%C3%BC%C5%9F-r.png"/>
-    <hyperlink ref="F10" r:id="rId2" display="https://ansiklopedi.subadapcocuk.org/images/thumb/d/d3/Dinonun_%C5%9Fark%C4%B1s%C4%B1_R.png/300px-Dinonun_%C5%9Fark%C4%B1s%C4%B1_R.png?20200628141720"/>
-    <hyperlink ref="D41" r:id="rId3" display="https://ansiklopedi.subadapcocuk.org/index.php/Ne%C5%9Feli_Bir_G%C3%BCn"/>
-    <hyperlink ref="F41" r:id="rId4" display="https://ansiklopedi.subadapcocuk.org/images/thumb/7/73/Ne%C5%9Feli_bi_g%C3%BCn.jpg/300px-Ne%C5%9Feli_bi_g%C3%BCn.jpg"/>
-    <hyperlink ref="D42" r:id="rId5" display="https://ansiklopedi.subadapcocuk.org/index.php/D%C3%BCnyan%C4%B1n_Do%C4%9Fum_G%C3%BCn%C3%BC"/>
-    <hyperlink ref="E42" r:id="rId6" display="https://ansiklopedi.subadapcocuk.org/images/d/d3/D%C3%BCnyan%C4%B1n_do%C4%9Fum_g%C3%BCn%C3%BC.mp3"/>
-    <hyperlink ref="F42" r:id="rId7" display="https://ansiklopedi.subadapcocuk.org/images/thumb/5/5b/D%C3%BCnyan%C4%B1n_do%C4%9Fum_g%C3%BCn%C3%BC_g%C3%B6rsel.jpg/300px-D%C3%BCnyan%C4%B1n_do%C4%9Fum_g%C3%BCn%C3%BC_g%C3%B6rsel.jpg"/>
-    <hyperlink ref="D43" r:id="rId8" display="https://ansiklopedi.subadapcocuk.org/index.php/Okul_Neresi%3F"/>
-    <hyperlink ref="F43" r:id="rId9" display="https://ansiklopedi.subadapcocuk.org/images/thumb/c/c3/Okul_Neresi%3F_G%C3%B6rsel.jpg/300px-Okul_Neresi%3F_G%C3%B6rsel.jpg"/>
-    <hyperlink ref="D44" r:id="rId10" display="https://ansiklopedi.subadapcocuk.org/index.php/En_%C4%B0yisi_De%C4%9Fil!"/>
-    <hyperlink ref="F44" r:id="rId11" display="https://ansiklopedi.subadapcocuk.org/images/thumb/e/e6/En_%C4%B0yisi_De%C4%9Fil.jpg/300px-En_%C4%B0yisi_De%C4%9Fil.jpg"/>
-    <hyperlink ref="D45" r:id="rId12" display="https://ansiklopedi.subadapcocuk.org/index.php/Bir_%C5%9Eiir_Yazd%C4%B1m"/>
-    <hyperlink ref="E45" r:id="rId13" display="https://ansiklopedi.subadapcocuk.org/images/c/ca/Bir_%C5%9Fiir_yazd%C4%B1m.mp3"/>
-    <hyperlink ref="F45" r:id="rId14" display="https://ansiklopedi.subadapcocuk.org/images/thumb/d/d3/Bir_%C5%9Fiir_Yazd%C4%B1m_G%C3%B6rsel.jpg/300px-Bir_%C5%9Fiir_Yazd%C4%B1m_G%C3%B6rsel.jpg"/>
-    <hyperlink ref="D46" r:id="rId15" display="https://ansiklopedi.subadapcocuk.org/index.php/%C3%87ocuk_Halay%C4%B1"/>
-    <hyperlink ref="E46" r:id="rId16" display="https://ansiklopedi.subadapcocuk.org/images/9/96/%C3%87ocuk_halay%C4%B1.mp3"/>
-    <hyperlink ref="F46" r:id="rId17" display="https://ansiklopedi.subadapcocuk.org/images/thumb/4/4d/%C3%87ocuk_halay%C4%B1_g%C3%B6rsel.jpg/300px-%C3%87ocuk_halay%C4%B1_g%C3%B6rsel.jpg"/>
-    <hyperlink ref="D47" r:id="rId18" display="https://ansiklopedi.subadapcocuk.org/index.php/Suzi"/>
-    <hyperlink ref="E47" r:id="rId19" display="https://ansiklopedi.subadapcocuk.org/images/3/31/Suzi.mp3"/>
-    <hyperlink ref="F47" r:id="rId20" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
-    <hyperlink ref="D48" r:id="rId21" display="https://ansiklopedi.subadapcocuk.org/index.php/Tak_Tak_Tak"/>
-    <hyperlink ref="E48" r:id="rId22" display="https://ansiklopedi.subadapcocuk.org/images/9/96/Tak_Tak_Tak.mp3"/>
-    <hyperlink ref="F48" r:id="rId23" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
-    <hyperlink ref="D49" r:id="rId24" display="https://ansiklopedi.subadapcocuk.org/index.php/%C5%9Ea%C5%9F%C4%B1ran_Mevsimler"/>
-    <hyperlink ref="E49" r:id="rId25" display="https://ansiklopedi.subadapcocuk.org/images/c/c4/%C5%9Ea%C5%9F%C4%B1ran_Mevsimler.mp3"/>
-    <hyperlink ref="F49" r:id="rId26" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
-    <hyperlink ref="D50" r:id="rId27" display="https://ansiklopedi.subadapcocuk.org/index.php/Evdeki_Hayalet"/>
-    <hyperlink ref="E50" r:id="rId28" display="https://ansiklopedi.subadapcocuk.org/images/0/0b/Evdeki_Hayalet.mp3"/>
-    <hyperlink ref="F50" r:id="rId29" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
-    <hyperlink ref="D51" r:id="rId30" display="https://ansiklopedi.subadapcocuk.org/index.php/Tak%C4%B1l_Kitaplar%C4%B1n_Kanatlar%C4%B1na"/>
-    <hyperlink ref="E51" r:id="rId31" display="https://ansiklopedi.subadapcocuk.org/images/f/f8/Tak%C4%B1l_Kitaplar%C4%B1n_Kanatlar%C4%B1na.mp3"/>
-    <hyperlink ref="F51" r:id="rId32" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
-    <hyperlink ref="D52" r:id="rId33" display="https://ansiklopedi.subadapcocuk.org/index.php/%C3%96c%C3%BC_M%C3%B6c%C3%BC_Yok_Ki"/>
-    <hyperlink ref="E52" r:id="rId34" display="https://ansiklopedi.subadapcocuk.org/images/9/9a/%C3%96c%C3%BC_M%C3%B6c%C3%BC_Yok_Ki.mp3"/>
-    <hyperlink ref="F52" r:id="rId35" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
+    <hyperlink ref="C2" r:id="rId1" display="Bilmiş Çocuğun Şarkıları"/>
+    <hyperlink ref="G2" r:id="rId2" display="https://ansiklopedi.subadapcocuk.org/images/thumb/e/e9/D%C3%BC%C5%9F-r.png/300px-D%C3%BC%C5%9F-r.png"/>
+    <hyperlink ref="C4" r:id="rId3" display="Bilmiş Çocuğun Şarkıları"/>
+    <hyperlink ref="C5" r:id="rId4" display="Bilmiş Çocuğun Şarkıları"/>
+    <hyperlink ref="C6" r:id="rId5" display="Bilmiş Çocuğun Şarkıları"/>
+    <hyperlink ref="C7" r:id="rId6" display="Bilmiş Çocuğun Şarkıları"/>
+    <hyperlink ref="G10" r:id="rId7" display="https://ansiklopedi.subadapcocuk.org/images/thumb/d/d3/Dinonun_%C5%9Fark%C4%B1s%C4%B1_R.png/300px-Dinonun_%C5%9Fark%C4%B1s%C4%B1_R.png?20200628141720"/>
+    <hyperlink ref="E41" r:id="rId8" display="https://ansiklopedi.subadapcocuk.org/index.php/Ne%C5%9Feli_Bir_G%C3%BCn"/>
+    <hyperlink ref="G41" r:id="rId9" display="https://ansiklopedi.subadapcocuk.org/images/thumb/7/73/Ne%C5%9Feli_bi_g%C3%BCn.jpg/300px-Ne%C5%9Feli_bi_g%C3%BCn.jpg"/>
+    <hyperlink ref="E42" r:id="rId10" display="https://ansiklopedi.subadapcocuk.org/index.php/D%C3%BCnyan%C4%B1n_Do%C4%9Fum_G%C3%BCn%C3%BC"/>
+    <hyperlink ref="F42" r:id="rId11" display="https://ansiklopedi.subadapcocuk.org/images/d/d3/D%C3%BCnyan%C4%B1n_do%C4%9Fum_g%C3%BCn%C3%BC.mp3"/>
+    <hyperlink ref="G42" r:id="rId12" display="https://ansiklopedi.subadapcocuk.org/images/thumb/5/5b/D%C3%BCnyan%C4%B1n_do%C4%9Fum_g%C3%BCn%C3%BC_g%C3%B6rsel.jpg/300px-D%C3%BCnyan%C4%B1n_do%C4%9Fum_g%C3%BCn%C3%BC_g%C3%B6rsel.jpg"/>
+    <hyperlink ref="E43" r:id="rId13" display="https://ansiklopedi.subadapcocuk.org/index.php/Okul_Neresi%3F"/>
+    <hyperlink ref="G43" r:id="rId14" display="https://ansiklopedi.subadapcocuk.org/images/thumb/c/c3/Okul_Neresi%3F_G%C3%B6rsel.jpg/300px-Okul_Neresi%3F_G%C3%B6rsel.jpg"/>
+    <hyperlink ref="E44" r:id="rId15" display="https://ansiklopedi.subadapcocuk.org/index.php/En_%C4%B0yisi_De%C4%9Fil!"/>
+    <hyperlink ref="G44" r:id="rId16" display="https://ansiklopedi.subadapcocuk.org/images/thumb/e/e6/En_%C4%B0yisi_De%C4%9Fil.jpg/300px-En_%C4%B0yisi_De%C4%9Fil.jpg"/>
+    <hyperlink ref="E45" r:id="rId17" display="https://ansiklopedi.subadapcocuk.org/index.php/Bir_%C5%9Eiir_Yazd%C4%B1m"/>
+    <hyperlink ref="F45" r:id="rId18" display="https://ansiklopedi.subadapcocuk.org/images/c/ca/Bir_%C5%9Fiir_yazd%C4%B1m.mp3"/>
+    <hyperlink ref="G45" r:id="rId19" display="https://ansiklopedi.subadapcocuk.org/images/thumb/d/d3/Bir_%C5%9Fiir_Yazd%C4%B1m_G%C3%B6rsel.jpg/300px-Bir_%C5%9Fiir_Yazd%C4%B1m_G%C3%B6rsel.jpg"/>
+    <hyperlink ref="E46" r:id="rId20" display="https://ansiklopedi.subadapcocuk.org/index.php/%C3%87ocuk_Halay%C4%B1"/>
+    <hyperlink ref="F46" r:id="rId21" display="https://ansiklopedi.subadapcocuk.org/images/9/96/%C3%87ocuk_halay%C4%B1.mp3"/>
+    <hyperlink ref="G46" r:id="rId22" display="https://ansiklopedi.subadapcocuk.org/images/thumb/4/4d/%C3%87ocuk_halay%C4%B1_g%C3%B6rsel.jpg/300px-%C3%87ocuk_halay%C4%B1_g%C3%B6rsel.jpg"/>
+    <hyperlink ref="E47" r:id="rId23" display="https://ansiklopedi.subadapcocuk.org/index.php/Suzi"/>
+    <hyperlink ref="F47" r:id="rId24" display="https://ansiklopedi.subadapcocuk.org/images/3/31/Suzi.mp3"/>
+    <hyperlink ref="G47" r:id="rId25" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
+    <hyperlink ref="E48" r:id="rId26" display="https://ansiklopedi.subadapcocuk.org/index.php/Tak_Tak_Tak"/>
+    <hyperlink ref="F48" r:id="rId27" display="https://ansiklopedi.subadapcocuk.org/images/9/96/Tak_Tak_Tak.mp3"/>
+    <hyperlink ref="G48" r:id="rId28" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
+    <hyperlink ref="E49" r:id="rId29" display="https://ansiklopedi.subadapcocuk.org/index.php/%C5%9Ea%C5%9F%C4%B1ran_Mevsimler"/>
+    <hyperlink ref="F49" r:id="rId30" display="https://ansiklopedi.subadapcocuk.org/images/c/c4/%C5%9Ea%C5%9F%C4%B1ran_Mevsimler.mp3"/>
+    <hyperlink ref="G49" r:id="rId31" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
+    <hyperlink ref="E50" r:id="rId32" display="https://ansiklopedi.subadapcocuk.org/index.php/Evdeki_Hayalet"/>
+    <hyperlink ref="F50" r:id="rId33" display="https://ansiklopedi.subadapcocuk.org/images/0/0b/Evdeki_Hayalet.mp3"/>
+    <hyperlink ref="G50" r:id="rId34" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
+    <hyperlink ref="E51" r:id="rId35" display="https://ansiklopedi.subadapcocuk.org/index.php/Tak%C4%B1l_Kitaplar%C4%B1n_Kanatlar%C4%B1na"/>
+    <hyperlink ref="F51" r:id="rId36" display="https://ansiklopedi.subadapcocuk.org/images/f/f8/Tak%C4%B1l_Kitaplar%C4%B1n_Kanatlar%C4%B1na.mp3"/>
+    <hyperlink ref="G51" r:id="rId37" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
+    <hyperlink ref="E52" r:id="rId38" display="https://ansiklopedi.subadapcocuk.org/index.php/%C3%96c%C3%BC_M%C3%B6c%C3%BC_Yok_Ki!"/>
+    <hyperlink ref="F52" r:id="rId39" display="https://ansiklopedi.subadapcocuk.org/images/9/9a/%C3%96c%C3%BC_M%C3%B6c%C3%BC_Yok_Ki.mp3"/>
+    <hyperlink ref="G52" r:id="rId40" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
[#43] Update Expo SDK to v55 and modernize audio playback (#96)
</commit_message>
<xml_diff>
--- a/data/subadapp.xlsx
+++ b/data/subadapp.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="228">
   <si>
     <t xml:space="preserve">no</t>
   </si>
@@ -113,6 +113,9 @@
     <t xml:space="preserve">albumNo</t>
   </si>
   <si>
+    <t xml:space="preserve">album</t>
+  </si>
+  <si>
     <t xml:space="preserve">url</t>
   </si>
   <si>
@@ -188,6 +191,9 @@
     <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/images/thumb/4/4a/%C5%9Eubadap_R.png/300px-%C5%9Eubadap_R.png</t>
   </si>
   <si>
+    <t xml:space="preserve"> Dino'nun Şarkıları</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ben Doğmadan Önce</t>
   </si>
   <si>
@@ -695,25 +701,7 @@
     <t xml:space="preserve">Öcü Möcü Yok Ki! </t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/index.php/%C3%96c%C3%BC_M%C3%B6c%C3%BC_Yok_Ki</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">!</t>
-    </r>
+    <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/index.php/%C3%96c%C3%BC_M%C3%B6c%C3%BC_Yok_Ki!</t>
   </si>
   <si>
     <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/images/9/9a/%C3%96c%C3%BC_M%C3%B6c%C3%BC_Yok_Ki.mp3</t>
@@ -726,7 +714,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -767,15 +755,20 @@
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -829,16 +822,20 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -846,11 +843,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1105,29 +1106,29 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="11.5625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5625" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="28.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="110.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="117.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="110.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="117.56"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1135,16 +1136,16 @@
       <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>2014</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1152,16 +1153,16 @@
       <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>2015</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="2" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1169,16 +1170,16 @@
       <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>2016</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1186,16 +1187,16 @@
       <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>2017</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="2" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1203,16 +1204,16 @@
       <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C6" s="1" t="n">
         <v>2019</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="4" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1220,16 +1221,16 @@
       <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C7" s="1" t="n">
         <v>2020</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" s="2" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1237,16 +1238,16 @@
       <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C8" s="1" t="n">
         <v>2023</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1254,16 +1255,16 @@
       <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C9" s="1" t="n">
         <v>2024</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E9" s="0" t="s">
+      <c r="E9" s="2" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1292,34 +1293,38 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
-  <sheetFormatPr defaultColWidth="11.5625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G52"/>
+  <sheetFormatPr defaultColWidth="11.5625" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3.76"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="102.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="135.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="200.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="28.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="25.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="102.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="135.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="200.11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1330,17 +1335,20 @@
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="D2" s="0" t="s">
+      <c r="C2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>34</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1351,16 +1359,19 @@
         <v>1</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="D3" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="2" t="s">
         <v>38</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1370,17 +1381,20 @@
       <c r="B4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="0" t="s">
-        <v>39</v>
-      </c>
-      <c r="D4" s="0" t="s">
+      <c r="C4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" s="2" t="s">
         <v>42</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1390,17 +1404,20 @@
       <c r="B5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="0" t="s">
-        <v>43</v>
-      </c>
-      <c r="D5" s="0" t="s">
+      <c r="C5" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" s="2" t="s">
         <v>46</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1410,17 +1427,20 @@
       <c r="B6" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="0" t="s">
-        <v>47</v>
-      </c>
-      <c r="D6" s="0" t="s">
+      <c r="C6" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" s="2" t="s">
         <v>50</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1430,17 +1450,20 @@
       <c r="B7" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="0" t="s">
-        <v>51</v>
-      </c>
-      <c r="D7" s="0" t="s">
+      <c r="C7" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="F7" s="0" t="s">
+      <c r="F7" s="2" t="s">
         <v>54</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1450,17 +1473,20 @@
       <c r="B8" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="D8" s="0" t="s">
+      <c r="C8" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="D8" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="F8" s="0" t="s">
+      <c r="E8" s="2" t="s">
         <v>58</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1470,17 +1496,20 @@
       <c r="B9" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="0" t="s">
-        <v>59</v>
-      </c>
-      <c r="D9" s="0" t="s">
-        <v>60</v>
-      </c>
-      <c r="E9" s="0" t="s">
+      <c r="C9" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F9" s="0" t="s">
+      <c r="E9" s="2" t="s">
         <v>62</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1490,17 +1519,20 @@
       <c r="B10" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="0" t="s">
-        <v>63</v>
-      </c>
-      <c r="D10" s="0" t="s">
-        <v>64</v>
-      </c>
-      <c r="E10" s="0" t="s">
+      <c r="C10" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="E10" s="2" t="s">
         <v>66</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1510,17 +1542,20 @@
       <c r="B11" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C11" s="0" t="s">
-        <v>67</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="E11" s="0" t="s">
+      <c r="C11" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F11" s="0" t="s">
+      <c r="E11" s="2" t="s">
         <v>70</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1530,17 +1565,20 @@
       <c r="B12" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="0" t="s">
-        <v>71</v>
-      </c>
-      <c r="D12" s="0" t="s">
-        <v>72</v>
-      </c>
-      <c r="E12" s="0" t="s">
+      <c r="C12" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="F12" s="0" t="s">
+      <c r="E12" s="2" t="s">
         <v>74</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1550,17 +1588,20 @@
       <c r="B13" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="0" t="s">
-        <v>75</v>
-      </c>
-      <c r="D13" s="0" t="s">
-        <v>76</v>
-      </c>
-      <c r="E13" s="0" t="s">
+      <c r="C13" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="F13" s="0" t="s">
+      <c r="E13" s="2" t="s">
         <v>78</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1570,17 +1611,20 @@
       <c r="B14" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="D14" s="0" t="s">
-        <v>80</v>
-      </c>
-      <c r="E14" s="0" t="s">
+      <c r="C14" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="F14" s="0" t="s">
+      <c r="E14" s="2" t="s">
         <v>82</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1590,17 +1634,20 @@
       <c r="B15" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="0" t="s">
-        <v>83</v>
-      </c>
-      <c r="D15" s="0" t="s">
-        <v>84</v>
-      </c>
-      <c r="E15" s="0" t="s">
+      <c r="C15" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F15" s="0" t="s">
+      <c r="E15" s="2" t="s">
         <v>86</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1610,17 +1657,20 @@
       <c r="B16" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C16" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="D16" s="0" t="s">
-        <v>88</v>
-      </c>
-      <c r="E16" s="0" t="s">
+      <c r="C16" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="F16" s="0" t="s">
+      <c r="E16" s="2" t="s">
         <v>90</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1630,17 +1680,20 @@
       <c r="B17" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C17" s="0" t="s">
-        <v>91</v>
-      </c>
-      <c r="D17" s="0" t="s">
-        <v>92</v>
-      </c>
-      <c r="E17" s="0" t="s">
+      <c r="C17" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="F17" s="0" t="s">
+      <c r="E17" s="2" t="s">
         <v>94</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1650,17 +1703,20 @@
       <c r="B18" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C18" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="D18" s="0" t="s">
-        <v>96</v>
-      </c>
-      <c r="E18" s="0" t="s">
+      <c r="C18" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="F18" s="0" t="s">
+      <c r="E18" s="2" t="s">
         <v>98</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1670,17 +1726,20 @@
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C19" s="0" t="s">
-        <v>99</v>
-      </c>
-      <c r="D19" s="0" t="s">
-        <v>100</v>
-      </c>
-      <c r="E19" s="0" t="s">
+      <c r="C19" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F19" s="0" t="s">
+      <c r="E19" s="2" t="s">
         <v>102</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1690,17 +1749,20 @@
       <c r="B20" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C20" s="0" t="s">
-        <v>103</v>
-      </c>
-      <c r="D20" s="0" t="s">
-        <v>104</v>
-      </c>
-      <c r="E20" s="0" t="s">
+      <c r="C20" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="F20" s="0" t="s">
+      <c r="E20" s="2" t="s">
         <v>106</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1710,17 +1772,20 @@
       <c r="B21" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="C21" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D21" s="0" t="s">
-        <v>107</v>
-      </c>
-      <c r="E21" s="0" t="s">
-        <v>108</v>
-      </c>
-      <c r="F21" s="0" t="s">
+      <c r="D21" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>109</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1730,17 +1795,20 @@
       <c r="B22" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C22" s="0" t="s">
-        <v>110</v>
-      </c>
-      <c r="D22" s="0" t="s">
-        <v>111</v>
-      </c>
-      <c r="E22" s="0" t="s">
+      <c r="C22" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="F22" s="0" t="s">
+      <c r="E22" s="2" t="s">
         <v>113</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1750,17 +1818,20 @@
       <c r="B23" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C23" s="0" t="s">
-        <v>114</v>
-      </c>
-      <c r="D23" s="0" t="s">
-        <v>115</v>
-      </c>
-      <c r="E23" s="0" t="s">
+      <c r="C23" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="F23" s="0" t="s">
+      <c r="E23" s="2" t="s">
         <v>117</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1770,17 +1841,20 @@
       <c r="B24" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C24" s="0" t="s">
-        <v>118</v>
-      </c>
-      <c r="D24" s="0" t="s">
-        <v>119</v>
-      </c>
-      <c r="E24" s="0" t="s">
+      <c r="C24" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="F24" s="0" t="s">
+      <c r="E24" s="2" t="s">
         <v>121</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1790,17 +1864,20 @@
       <c r="B25" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C25" s="0" t="s">
-        <v>122</v>
-      </c>
-      <c r="D25" s="0" t="s">
-        <v>123</v>
-      </c>
-      <c r="E25" s="0" t="s">
+      <c r="C25" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F25" s="0" t="s">
+      <c r="E25" s="2" t="s">
         <v>125</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1810,17 +1887,20 @@
       <c r="B26" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C26" s="0" t="s">
-        <v>126</v>
-      </c>
-      <c r="D26" s="0" t="s">
-        <v>127</v>
-      </c>
-      <c r="E26" s="0" t="s">
+      <c r="C26" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="F26" s="0" t="s">
+      <c r="E26" s="2" t="s">
         <v>129</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1830,17 +1910,20 @@
       <c r="B27" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C27" s="0" t="s">
-        <v>130</v>
-      </c>
-      <c r="D27" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="E27" s="0" t="s">
+      <c r="C27" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="F27" s="0" t="s">
+      <c r="E27" s="2" t="s">
         <v>133</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1850,17 +1933,20 @@
       <c r="B28" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C28" s="0" t="s">
+      <c r="C28" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D28" s="0" t="s">
-        <v>134</v>
-      </c>
-      <c r="E28" s="0" t="s">
-        <v>135</v>
-      </c>
-      <c r="F28" s="0" t="s">
+      <c r="D28" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>136</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1870,17 +1956,20 @@
       <c r="B29" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C29" s="0" t="s">
-        <v>137</v>
-      </c>
-      <c r="D29" s="0" t="s">
-        <v>138</v>
-      </c>
-      <c r="E29" s="0" t="s">
+      <c r="C29" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="F29" s="0" t="s">
+      <c r="E29" s="2" t="s">
         <v>140</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1890,17 +1979,20 @@
       <c r="B30" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C30" s="0" t="s">
-        <v>141</v>
-      </c>
-      <c r="D30" s="0" t="s">
-        <v>142</v>
-      </c>
-      <c r="E30" s="0" t="s">
+      <c r="C30" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F30" s="0" t="s">
+      <c r="E30" s="2" t="s">
         <v>144</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1910,17 +2002,20 @@
       <c r="B31" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C31" s="0" t="s">
-        <v>145</v>
-      </c>
-      <c r="D31" s="0" t="s">
-        <v>146</v>
-      </c>
-      <c r="E31" s="0" t="s">
+      <c r="C31" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="F31" s="0" t="s">
+      <c r="E31" s="2" t="s">
         <v>148</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1930,17 +2025,20 @@
       <c r="B32" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C32" s="0" t="s">
-        <v>149</v>
-      </c>
-      <c r="D32" s="0" t="s">
-        <v>150</v>
-      </c>
-      <c r="E32" s="0" t="s">
+      <c r="C32" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D32" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="F32" s="0" t="s">
+      <c r="E32" s="2" t="s">
         <v>152</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1950,17 +2048,20 @@
       <c r="B33" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C33" s="0" t="s">
+      <c r="C33" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D33" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="E33" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="F33" s="0" t="s">
+      <c r="D33" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>155</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1970,17 +2071,20 @@
       <c r="B34" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C34" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="D34" s="0" t="s">
-        <v>157</v>
-      </c>
-      <c r="E34" s="0" t="s">
+      <c r="C34" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D34" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="F34" s="0" t="s">
+      <c r="E34" s="2" t="s">
         <v>159</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1990,17 +2094,20 @@
       <c r="B35" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C35" s="0" t="s">
-        <v>160</v>
-      </c>
-      <c r="D35" s="0" t="s">
-        <v>161</v>
-      </c>
-      <c r="E35" s="0" t="s">
+      <c r="C35" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="F35" s="0" t="s">
+      <c r="E35" s="2" t="s">
         <v>163</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2010,17 +2117,20 @@
       <c r="B36" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C36" s="0" t="s">
-        <v>164</v>
-      </c>
-      <c r="D36" s="0" t="s">
-        <v>165</v>
-      </c>
-      <c r="E36" s="0" t="s">
+      <c r="C36" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="F36" s="0" t="s">
+      <c r="E36" s="2" t="s">
         <v>167</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2030,17 +2140,20 @@
       <c r="B37" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C37" s="0" t="s">
-        <v>168</v>
-      </c>
-      <c r="D37" s="0" t="s">
-        <v>169</v>
-      </c>
-      <c r="E37" s="0" t="s">
+      <c r="C37" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D37" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="F37" s="0" t="s">
+      <c r="E37" s="2" t="s">
         <v>171</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2050,17 +2163,20 @@
       <c r="B38" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C38" s="0" t="s">
-        <v>172</v>
-      </c>
-      <c r="D38" s="0" t="s">
-        <v>173</v>
-      </c>
-      <c r="E38" s="0" t="s">
+      <c r="C38" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="F38" s="0" t="s">
+      <c r="E38" s="2" t="s">
         <v>175</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2070,17 +2186,20 @@
       <c r="B39" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C39" s="0" t="s">
-        <v>176</v>
-      </c>
-      <c r="D39" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="E39" s="0" t="s">
+      <c r="C39" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="F39" s="0" t="s">
+      <c r="E39" s="2" t="s">
         <v>179</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2090,17 +2209,20 @@
       <c r="B40" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C40" s="0" t="s">
-        <v>180</v>
-      </c>
-      <c r="D40" s="0" t="s">
-        <v>181</v>
-      </c>
-      <c r="E40" s="0" t="s">
+      <c r="C40" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="F40" s="0" t="s">
+      <c r="E40" s="2" t="s">
         <v>183</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2110,17 +2232,20 @@
       <c r="B41" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C41" s="0" t="s">
-        <v>184</v>
-      </c>
-      <c r="D41" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="E41" s="0" t="s">
+      <c r="C41" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D41" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="F41" s="3" t="s">
+      <c r="E41" s="4" t="s">
         <v>187</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2130,17 +2255,20 @@
       <c r="B42" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C42" s="0" t="s">
-        <v>188</v>
-      </c>
-      <c r="D42" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="E42" s="3" t="s">
+      <c r="C42" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D42" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="F42" s="3" t="s">
+      <c r="E42" s="4" t="s">
         <v>191</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2150,17 +2278,20 @@
       <c r="B43" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C43" s="0" t="s">
-        <v>192</v>
-      </c>
-      <c r="D43" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="E43" s="0" t="s">
+      <c r="C43" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D43" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="F43" s="3" t="s">
+      <c r="E43" s="4" t="s">
         <v>195</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2170,17 +2301,20 @@
       <c r="B44" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C44" s="0" t="s">
-        <v>196</v>
-      </c>
-      <c r="D44" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="E44" s="0" t="s">
+      <c r="C44" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D44" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="F44" s="3" t="s">
+      <c r="E44" s="4" t="s">
         <v>199</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="G44" s="4" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2190,17 +2324,20 @@
       <c r="B45" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C45" s="0" t="s">
-        <v>200</v>
-      </c>
-      <c r="D45" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="E45" s="3" t="s">
+      <c r="C45" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="F45" s="3" t="s">
+      <c r="E45" s="4" t="s">
         <v>203</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2210,17 +2347,20 @@
       <c r="B46" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C46" s="0" t="s">
-        <v>204</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="E46" s="3" t="s">
+      <c r="C46" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D46" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="F46" s="3" t="s">
+      <c r="E46" s="4" t="s">
         <v>207</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="G46" s="4" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2230,16 +2370,19 @@
       <c r="B47" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C47" s="0" t="s">
-        <v>208</v>
-      </c>
-      <c r="D47" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="E47" s="4" t="s">
+      <c r="C47" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D47" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="F47" s="5" t="s">
+      <c r="E47" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G47" s="7" t="s">
         <v>28</v>
       </c>
     </row>
@@ -2250,16 +2393,19 @@
       <c r="B48" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C48" s="0" t="s">
-        <v>211</v>
-      </c>
-      <c r="D48" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="E48" s="4" t="s">
+      <c r="C48" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D48" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="F48" s="5" t="s">
+      <c r="E48" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="F48" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="G48" s="7" t="s">
         <v>28</v>
       </c>
     </row>
@@ -2270,16 +2416,19 @@
       <c r="B49" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C49" s="0" t="s">
-        <v>214</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="E49" s="4" t="s">
+      <c r="C49" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D49" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="F49" s="5" t="s">
+      <c r="E49" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="F49" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="G49" s="7" t="s">
         <v>28</v>
       </c>
     </row>
@@ -2290,16 +2439,19 @@
       <c r="B50" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C50" s="0" t="s">
-        <v>217</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="E50" s="4" t="s">
+      <c r="C50" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D50" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="F50" s="5" t="s">
+      <c r="E50" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="F50" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="G50" s="7" t="s">
         <v>28</v>
       </c>
     </row>
@@ -2310,16 +2462,19 @@
       <c r="B51" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C51" s="0" t="s">
-        <v>220</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="E51" s="4" t="s">
+      <c r="C51" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D51" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="F51" s="5" t="s">
+      <c r="E51" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="G51" s="7" t="s">
         <v>28</v>
       </c>
     </row>
@@ -2330,56 +2485,64 @@
       <c r="B52" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C52" s="0" t="s">
-        <v>223</v>
-      </c>
-      <c r="D52" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="E52" s="4" t="s">
+      <c r="C52" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="F52" s="5" t="s">
+      <c r="E52" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="F52" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="G52" s="7" t="s">
         <v>28</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" display="https://ansiklopedi.subadapcocuk.org/images/thumb/e/e9/D%C3%BC%C5%9F-r.png/300px-D%C3%BC%C5%9F-r.png"/>
-    <hyperlink ref="F10" r:id="rId2" display="https://ansiklopedi.subadapcocuk.org/images/thumb/d/d3/Dinonun_%C5%9Fark%C4%B1s%C4%B1_R.png/300px-Dinonun_%C5%9Fark%C4%B1s%C4%B1_R.png?20200628141720"/>
-    <hyperlink ref="D41" r:id="rId3" display="https://ansiklopedi.subadapcocuk.org/index.php/Ne%C5%9Feli_Bir_G%C3%BCn"/>
-    <hyperlink ref="F41" r:id="rId4" display="https://ansiklopedi.subadapcocuk.org/images/thumb/7/73/Ne%C5%9Feli_bi_g%C3%BCn.jpg/300px-Ne%C5%9Feli_bi_g%C3%BCn.jpg"/>
-    <hyperlink ref="D42" r:id="rId5" display="https://ansiklopedi.subadapcocuk.org/index.php/D%C3%BCnyan%C4%B1n_Do%C4%9Fum_G%C3%BCn%C3%BC"/>
-    <hyperlink ref="E42" r:id="rId6" display="https://ansiklopedi.subadapcocuk.org/images/d/d3/D%C3%BCnyan%C4%B1n_do%C4%9Fum_g%C3%BCn%C3%BC.mp3"/>
-    <hyperlink ref="F42" r:id="rId7" display="https://ansiklopedi.subadapcocuk.org/images/thumb/5/5b/D%C3%BCnyan%C4%B1n_do%C4%9Fum_g%C3%BCn%C3%BC_g%C3%B6rsel.jpg/300px-D%C3%BCnyan%C4%B1n_do%C4%9Fum_g%C3%BCn%C3%BC_g%C3%B6rsel.jpg"/>
-    <hyperlink ref="D43" r:id="rId8" display="https://ansiklopedi.subadapcocuk.org/index.php/Okul_Neresi%3F"/>
-    <hyperlink ref="F43" r:id="rId9" display="https://ansiklopedi.subadapcocuk.org/images/thumb/c/c3/Okul_Neresi%3F_G%C3%B6rsel.jpg/300px-Okul_Neresi%3F_G%C3%B6rsel.jpg"/>
-    <hyperlink ref="D44" r:id="rId10" display="https://ansiklopedi.subadapcocuk.org/index.php/En_%C4%B0yisi_De%C4%9Fil!"/>
-    <hyperlink ref="F44" r:id="rId11" display="https://ansiklopedi.subadapcocuk.org/images/thumb/e/e6/En_%C4%B0yisi_De%C4%9Fil.jpg/300px-En_%C4%B0yisi_De%C4%9Fil.jpg"/>
-    <hyperlink ref="D45" r:id="rId12" display="https://ansiklopedi.subadapcocuk.org/index.php/Bir_%C5%9Eiir_Yazd%C4%B1m"/>
-    <hyperlink ref="E45" r:id="rId13" display="https://ansiklopedi.subadapcocuk.org/images/c/ca/Bir_%C5%9Fiir_yazd%C4%B1m.mp3"/>
-    <hyperlink ref="F45" r:id="rId14" display="https://ansiklopedi.subadapcocuk.org/images/thumb/d/d3/Bir_%C5%9Fiir_Yazd%C4%B1m_G%C3%B6rsel.jpg/300px-Bir_%C5%9Fiir_Yazd%C4%B1m_G%C3%B6rsel.jpg"/>
-    <hyperlink ref="D46" r:id="rId15" display="https://ansiklopedi.subadapcocuk.org/index.php/%C3%87ocuk_Halay%C4%B1"/>
-    <hyperlink ref="E46" r:id="rId16" display="https://ansiklopedi.subadapcocuk.org/images/9/96/%C3%87ocuk_halay%C4%B1.mp3"/>
-    <hyperlink ref="F46" r:id="rId17" display="https://ansiklopedi.subadapcocuk.org/images/thumb/4/4d/%C3%87ocuk_halay%C4%B1_g%C3%B6rsel.jpg/300px-%C3%87ocuk_halay%C4%B1_g%C3%B6rsel.jpg"/>
-    <hyperlink ref="D47" r:id="rId18" display="https://ansiklopedi.subadapcocuk.org/index.php/Suzi"/>
-    <hyperlink ref="E47" r:id="rId19" display="https://ansiklopedi.subadapcocuk.org/images/3/31/Suzi.mp3"/>
-    <hyperlink ref="F47" r:id="rId20" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
-    <hyperlink ref="D48" r:id="rId21" display="https://ansiklopedi.subadapcocuk.org/index.php/Tak_Tak_Tak"/>
-    <hyperlink ref="E48" r:id="rId22" display="https://ansiklopedi.subadapcocuk.org/images/9/96/Tak_Tak_Tak.mp3"/>
-    <hyperlink ref="F48" r:id="rId23" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
-    <hyperlink ref="D49" r:id="rId24" display="https://ansiklopedi.subadapcocuk.org/index.php/%C5%9Ea%C5%9F%C4%B1ran_Mevsimler"/>
-    <hyperlink ref="E49" r:id="rId25" display="https://ansiklopedi.subadapcocuk.org/images/c/c4/%C5%9Ea%C5%9F%C4%B1ran_Mevsimler.mp3"/>
-    <hyperlink ref="F49" r:id="rId26" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
-    <hyperlink ref="D50" r:id="rId27" display="https://ansiklopedi.subadapcocuk.org/index.php/Evdeki_Hayalet"/>
-    <hyperlink ref="E50" r:id="rId28" display="https://ansiklopedi.subadapcocuk.org/images/0/0b/Evdeki_Hayalet.mp3"/>
-    <hyperlink ref="F50" r:id="rId29" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
-    <hyperlink ref="D51" r:id="rId30" display="https://ansiklopedi.subadapcocuk.org/index.php/Tak%C4%B1l_Kitaplar%C4%B1n_Kanatlar%C4%B1na"/>
-    <hyperlink ref="E51" r:id="rId31" display="https://ansiklopedi.subadapcocuk.org/images/f/f8/Tak%C4%B1l_Kitaplar%C4%B1n_Kanatlar%C4%B1na.mp3"/>
-    <hyperlink ref="F51" r:id="rId32" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
-    <hyperlink ref="D52" r:id="rId33" display="https://ansiklopedi.subadapcocuk.org/index.php/%C3%96c%C3%BC_M%C3%B6c%C3%BC_Yok_Ki"/>
-    <hyperlink ref="E52" r:id="rId34" display="https://ansiklopedi.subadapcocuk.org/images/9/9a/%C3%96c%C3%BC_M%C3%B6c%C3%BC_Yok_Ki.mp3"/>
-    <hyperlink ref="F52" r:id="rId35" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
+    <hyperlink ref="C2" r:id="rId1" display="Bilmiş Çocuğun Şarkıları"/>
+    <hyperlink ref="G2" r:id="rId2" display="https://ansiklopedi.subadapcocuk.org/images/thumb/e/e9/D%C3%BC%C5%9F-r.png/300px-D%C3%BC%C5%9F-r.png"/>
+    <hyperlink ref="C4" r:id="rId3" display="Bilmiş Çocuğun Şarkıları"/>
+    <hyperlink ref="C5" r:id="rId4" display="Bilmiş Çocuğun Şarkıları"/>
+    <hyperlink ref="C6" r:id="rId5" display="Bilmiş Çocuğun Şarkıları"/>
+    <hyperlink ref="C7" r:id="rId6" display="Bilmiş Çocuğun Şarkıları"/>
+    <hyperlink ref="G10" r:id="rId7" display="https://ansiklopedi.subadapcocuk.org/images/thumb/d/d3/Dinonun_%C5%9Fark%C4%B1s%C4%B1_R.png/300px-Dinonun_%C5%9Fark%C4%B1s%C4%B1_R.png?20200628141720"/>
+    <hyperlink ref="E41" r:id="rId8" display="https://ansiklopedi.subadapcocuk.org/index.php/Ne%C5%9Feli_Bir_G%C3%BCn"/>
+    <hyperlink ref="G41" r:id="rId9" display="https://ansiklopedi.subadapcocuk.org/images/thumb/7/73/Ne%C5%9Feli_bi_g%C3%BCn.jpg/300px-Ne%C5%9Feli_bi_g%C3%BCn.jpg"/>
+    <hyperlink ref="E42" r:id="rId10" display="https://ansiklopedi.subadapcocuk.org/index.php/D%C3%BCnyan%C4%B1n_Do%C4%9Fum_G%C3%BCn%C3%BC"/>
+    <hyperlink ref="F42" r:id="rId11" display="https://ansiklopedi.subadapcocuk.org/images/d/d3/D%C3%BCnyan%C4%B1n_do%C4%9Fum_g%C3%BCn%C3%BC.mp3"/>
+    <hyperlink ref="G42" r:id="rId12" display="https://ansiklopedi.subadapcocuk.org/images/thumb/5/5b/D%C3%BCnyan%C4%B1n_do%C4%9Fum_g%C3%BCn%C3%BC_g%C3%B6rsel.jpg/300px-D%C3%BCnyan%C4%B1n_do%C4%9Fum_g%C3%BCn%C3%BC_g%C3%B6rsel.jpg"/>
+    <hyperlink ref="E43" r:id="rId13" display="https://ansiklopedi.subadapcocuk.org/index.php/Okul_Neresi%3F"/>
+    <hyperlink ref="G43" r:id="rId14" display="https://ansiklopedi.subadapcocuk.org/images/thumb/c/c3/Okul_Neresi%3F_G%C3%B6rsel.jpg/300px-Okul_Neresi%3F_G%C3%B6rsel.jpg"/>
+    <hyperlink ref="E44" r:id="rId15" display="https://ansiklopedi.subadapcocuk.org/index.php/En_%C4%B0yisi_De%C4%9Fil!"/>
+    <hyperlink ref="G44" r:id="rId16" display="https://ansiklopedi.subadapcocuk.org/images/thumb/e/e6/En_%C4%B0yisi_De%C4%9Fil.jpg/300px-En_%C4%B0yisi_De%C4%9Fil.jpg"/>
+    <hyperlink ref="E45" r:id="rId17" display="https://ansiklopedi.subadapcocuk.org/index.php/Bir_%C5%9Eiir_Yazd%C4%B1m"/>
+    <hyperlink ref="F45" r:id="rId18" display="https://ansiklopedi.subadapcocuk.org/images/c/ca/Bir_%C5%9Fiir_yazd%C4%B1m.mp3"/>
+    <hyperlink ref="G45" r:id="rId19" display="https://ansiklopedi.subadapcocuk.org/images/thumb/d/d3/Bir_%C5%9Fiir_Yazd%C4%B1m_G%C3%B6rsel.jpg/300px-Bir_%C5%9Fiir_Yazd%C4%B1m_G%C3%B6rsel.jpg"/>
+    <hyperlink ref="E46" r:id="rId20" display="https://ansiklopedi.subadapcocuk.org/index.php/%C3%87ocuk_Halay%C4%B1"/>
+    <hyperlink ref="F46" r:id="rId21" display="https://ansiklopedi.subadapcocuk.org/images/9/96/%C3%87ocuk_halay%C4%B1.mp3"/>
+    <hyperlink ref="G46" r:id="rId22" display="https://ansiklopedi.subadapcocuk.org/images/thumb/4/4d/%C3%87ocuk_halay%C4%B1_g%C3%B6rsel.jpg/300px-%C3%87ocuk_halay%C4%B1_g%C3%B6rsel.jpg"/>
+    <hyperlink ref="E47" r:id="rId23" display="https://ansiklopedi.subadapcocuk.org/index.php/Suzi"/>
+    <hyperlink ref="F47" r:id="rId24" display="https://ansiklopedi.subadapcocuk.org/images/3/31/Suzi.mp3"/>
+    <hyperlink ref="G47" r:id="rId25" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
+    <hyperlink ref="E48" r:id="rId26" display="https://ansiklopedi.subadapcocuk.org/index.php/Tak_Tak_Tak"/>
+    <hyperlink ref="F48" r:id="rId27" display="https://ansiklopedi.subadapcocuk.org/images/9/96/Tak_Tak_Tak.mp3"/>
+    <hyperlink ref="G48" r:id="rId28" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
+    <hyperlink ref="E49" r:id="rId29" display="https://ansiklopedi.subadapcocuk.org/index.php/%C5%9Ea%C5%9F%C4%B1ran_Mevsimler"/>
+    <hyperlink ref="F49" r:id="rId30" display="https://ansiklopedi.subadapcocuk.org/images/c/c4/%C5%9Ea%C5%9F%C4%B1ran_Mevsimler.mp3"/>
+    <hyperlink ref="G49" r:id="rId31" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
+    <hyperlink ref="E50" r:id="rId32" display="https://ansiklopedi.subadapcocuk.org/index.php/Evdeki_Hayalet"/>
+    <hyperlink ref="F50" r:id="rId33" display="https://ansiklopedi.subadapcocuk.org/images/0/0b/Evdeki_Hayalet.mp3"/>
+    <hyperlink ref="G50" r:id="rId34" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
+    <hyperlink ref="E51" r:id="rId35" display="https://ansiklopedi.subadapcocuk.org/index.php/Tak%C4%B1l_Kitaplar%C4%B1n_Kanatlar%C4%B1na"/>
+    <hyperlink ref="F51" r:id="rId36" display="https://ansiklopedi.subadapcocuk.org/images/f/f8/Tak%C4%B1l_Kitaplar%C4%B1n_Kanatlar%C4%B1na.mp3"/>
+    <hyperlink ref="G51" r:id="rId37" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
+    <hyperlink ref="E52" r:id="rId38" display="https://ansiklopedi.subadapcocuk.org/index.php/%C3%96c%C3%BC_M%C3%B6c%C3%BC_Yok_Ki!"/>
+    <hyperlink ref="F52" r:id="rId39" display="https://ansiklopedi.subadapcocuk.org/images/9/9a/%C3%96c%C3%BC_M%C3%B6c%C3%BC_Yok_Ki.mp3"/>
+    <hyperlink ref="G52" r:id="rId40" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>